<commit_message>
Add Americas, Europe, and Asia regional tabs to Gen AI market insights
Three new regional tabs, each with 5 sections:
- Leaders: Key executives and founders by region
- Companies with Most Momentum: Fastest-growing companies
- Biggest Breakthroughs: Region-specific innovations
- Top Investors: VCs, corporate, and angel investors
- Hotspots: Top cities and hubs

Americas: 7 leaders, 8 companies, 4 breakthroughs, 9 investors, 6 hotspots
Europe: 6 leaders, 6 companies, 4 breakthroughs, 8 investors, 6 hotspots
Asia: 8 leaders, 8 companies, 5 breakthroughs, 7 investors, 7 hotspots

Co-authored-by: ms4674 <ms4674@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/generative_ai_market_insights.xlsx
+++ b/generative_ai_market_insights.xlsx
@@ -13,6 +13,9 @@
     <sheet name="Best Investors" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Best Hotspots" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Summary Dashboard" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Americas" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Europe" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Asia" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -22,7 +25,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -38,8 +41,12 @@
     <font>
       <sz val="11"/>
     </font>
+    <font>
+      <b val="1"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -52,8 +59,20 @@
         <bgColor rgb="001F4E79"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002E75B6"/>
+        <bgColor rgb="002E75B6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D6E4F0"/>
+        <bgColor rgb="00D6E4F0"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -67,17 +86,53 @@
       <top style="thin"/>
       <bottom style="thin"/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin"/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2663,4 +2718,4519 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G48"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="35" customWidth="1" min="2" max="2"/>
+    <col width="29" customWidth="1" min="3" max="3"/>
+    <col width="38" customWidth="1" min="4" max="4"/>
+    <col width="50" customWidth="1" min="5" max="5"/>
+    <col width="50" customWidth="1" min="6" max="6"/>
+    <col width="50" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>LEADERS</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="n"/>
+      <c r="C1" s="4" t="n"/>
+      <c r="D1" s="4" t="n"/>
+      <c r="E1" s="4" t="n"/>
+      <c r="F1" s="4" t="n"/>
+      <c r="G1" s="5" t="n"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B2" s="6" t="inlineStr">
+        <is>
+          <t>Leader</t>
+        </is>
+      </c>
+      <c r="C2" s="6" t="inlineStr">
+        <is>
+          <t>Title / Company</t>
+        </is>
+      </c>
+      <c r="D2" s="6" t="inlineStr">
+        <is>
+          <t>HQ</t>
+        </is>
+      </c>
+      <c r="E2" s="6" t="inlineStr">
+        <is>
+          <t>Key Achievements (Past 12 Months)</t>
+        </is>
+      </c>
+      <c r="F2" s="6" t="inlineStr">
+        <is>
+          <t>Why They Stand Out</t>
+        </is>
+      </c>
+      <c r="G2" s="6" t="inlineStr">
+        <is>
+          <t>Recognition</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Sam Altman</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>CEO, OpenAI</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>San Francisco, CA</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>$110B funding at $840B valuation; GPT-5.4 agentic launch; 800-900M weekly users; preparing IPO</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Built the fastest-growing business platform in history; AGI research leader</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>TIME 100 AI 2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Jensen Huang</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>CEO, NVIDIA</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Santa Clara, CA</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>NVIDIA at $4T market cap; Nemotron 3 Super; GPUs power virtually all frontier AI</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Indispensable AI infrastructure — every major model trains on NVIDIA hardware</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>TIME 100 AI 2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Dario Amodei</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>CEO, Anthropic</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>San Francisco, CA</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>$30B Series G at $380B; $14B revenue; 10x annual growth 3 yrs; Claude 5 GPQA record</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>Safety-first frontier AI; Claude Code at $2.5B+ run-rate; 4% of GitHub public commits</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>TIME 100 AI 2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Satya Nadella</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Chairman &amp; CEO, Microsoft</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Redmond, WA</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Lead investor in OpenAI $110B; Azure AI expansion; Microsoft 365 Copilot at scale</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>Enterprise AI adoption at unprecedented scale</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>TIME 100 AI 2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Elon Musk</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>CEO, xAI / Tesla / SpaceX</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Austin, TX</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>xAI at ~$3.8B revenue (38x YoY); $20B Series E at $230B; merged with X platform</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>Massive compute investment; Grok models; ambitious AGI timeline</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>TIME 100 AI 2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Mustafa Suleyman</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>CEO, Microsoft AI</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Redmond, WA</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Leading Microsoft's AI product strategy; AI integration across consumer &amp; enterprise</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>DeepMind co-founder experience brought to Microsoft</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>TIME 100 AI 2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Sundar Pichai</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>CEO, Google / Alphabet</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Mountain View, CA</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>Gemini 3.1 Pro launch; AI integration across Search, Cloud, enterprise</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>Multi-model strategy across Google's massive product surface</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>TIME 100 AI 2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="10"/>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>COMPANIES WITH MOST MOMENTUM</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="n"/>
+      <c r="C11" s="4" t="n"/>
+      <c r="D11" s="4" t="n"/>
+      <c r="E11" s="4" t="n"/>
+      <c r="F11" s="4" t="n"/>
+      <c r="G11" s="5" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="inlineStr">
+        <is>
+          <t>HQ</t>
+        </is>
+      </c>
+      <c r="D12" s="6" t="inlineStr">
+        <is>
+          <t>Valuation</t>
+        </is>
+      </c>
+      <c r="E12" s="6" t="inlineStr">
+        <is>
+          <t>Revenue / Growth</t>
+        </is>
+      </c>
+      <c r="F12" s="6" t="inlineStr">
+        <is>
+          <t>Key Momentum Indicators</t>
+        </is>
+      </c>
+      <c r="G12" s="6" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>San Francisco, CA</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>$840B</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>800-900M weekly users; 2B daily prompts; 1M+ business customers</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>$110B funding round — largest private round in history; GPT-5.4 agentic launch</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>Foundation Model / Consumer + Enterprise</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Anthropic</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>San Francisco, CA</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>$380B</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>$14B annualized revenue; 10x growth 3 yrs; 300K+ business customers</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>Claude Code $2.5B+ run-rate; Claude 5 GPQA record; 8 of Fortune 10</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>Foundation Model / Enterprise AI</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>xAI</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Austin, TX</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>$230B</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>~$3.8B annualized revenue; 38x YoY</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>$20B Series E; merged with X platform; SuperGrok products</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>Foundation Model / Consumer AI</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Cursor (Anysphere)</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>San Francisco, CA</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>N/A (private)</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>$2B ARR in 18 months</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>Fastest revenue ramp in enterprise software history</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>AI-Native Developer Tool</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Perplexity</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>San Francisco, CA</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>$20B</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>$148M ARR; 800% YoY; targeting $656M by end-2026</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>30M monthly users; expanding into advertising &amp; commerce</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>AI Search / Consumer AI</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Scale AI</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>San Francisco, CA</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>$14.3B+</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>Leading AI training data provider</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>$14.3B Meta-led round; critical infrastructure for frontier models</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>AI Infrastructure / Data</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Cohere</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Toronto, Canada</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>~$5.5B</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>Growing enterprise customer base across financial services, healthcare</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>Enterprise AI with private deployment; strong Canadian AI ecosystem</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>Enterprise AI / NLP</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Adept</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>San Francisco, CA</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>~$1B+</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>Agentic AI for workforce automation</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>Building enterprise agents for complex workflows across applications</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>Agentic AI</t>
+        </is>
+      </c>
+    </row>
+    <row r="21"/>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>BIGGEST BREAKTHROUGHS</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="n"/>
+      <c r="C22" s="4" t="n"/>
+      <c r="D22" s="4" t="n"/>
+      <c r="E22" s="4" t="n"/>
+      <c r="F22" s="4" t="n"/>
+      <c r="G22" s="5" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="6" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B23" s="6" t="inlineStr">
+        <is>
+          <t>Breakthrough</t>
+        </is>
+      </c>
+      <c r="C23" s="6" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="D23" s="6" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="E23" s="6" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="F23" s="6" t="inlineStr">
+        <is>
+          <t>Impact</t>
+        </is>
+      </c>
+      <c r="G23" s="6" t="inlineStr">
+        <is>
+          <t>Technical Details</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>GPT-5.4 Autonomous Agents</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>Mar 2026</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>Native computer-use for autonomous agent workflows</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>Major step toward fully autonomous AI agents; 33% fewer false claims</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>Multi-source info gathering; agentic computer use; enterprise workflows</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>Claude 5 GPQA Diamond Record</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>Anthropic</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>Mar 2026</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>87.3% GPQA Diamond — first AI system to exceed 85%</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>8.1pp improvement; new frontier in scientific reasoning</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>Inference-time reasoning optimization; Extended Thinking mode (+15pp)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>NVIDIA Nemotron 3 Super</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>NVIDIA</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>2025-2026</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>120B-param open model; 5x throughput for agentic AI; 1M-token context</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>Prevents goal drift in multi-agent systems; major efficiency gain</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>Hybrid MoE; multi-token prediction; 3x faster inference</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>Gemini 3.1 Pro</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>Google DeepMind</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>Feb 2026</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>Advanced reasoning model for complex problem-solving &amp; agentic workflows</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>Keeps Google competitive in frontier model race</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>Multi-modal reasoning; improved tool use and planning</t>
+        </is>
+      </c>
+    </row>
+    <row r="28"/>
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>TOP INVESTORS</t>
+        </is>
+      </c>
+      <c r="B29" s="4" t="n"/>
+      <c r="C29" s="4" t="n"/>
+      <c r="D29" s="4" t="n"/>
+      <c r="E29" s="4" t="n"/>
+      <c r="F29" s="4" t="n"/>
+      <c r="G29" s="5" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="6" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B30" s="6" t="inlineStr">
+        <is>
+          <t>Investor / Firm</t>
+        </is>
+      </c>
+      <c r="C30" s="6" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="D30" s="6" t="inlineStr">
+        <is>
+          <t>HQ</t>
+        </is>
+      </c>
+      <c r="E30" s="6" t="inlineStr">
+        <is>
+          <t>Notable Gen AI Investments</t>
+        </is>
+      </c>
+      <c r="F30" s="6" t="inlineStr">
+        <is>
+          <t>Investment Thesis</t>
+        </is>
+      </c>
+      <c r="G30" s="6" t="inlineStr">
+        <is>
+          <t>Standout Metric</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>Strategic / Corporate</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>Seattle, WA</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>OpenAI ($50B in Feb 2026 round); AWS AI infrastructure</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>AI compute/infrastructure dominance via AWS</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>Largest single investor in OpenAI's $110B round</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>NVIDIA</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>Strategic / Corporate</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>Santa Clara, CA</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>OpenAI ($30B); AMI Labs; broad AI ecosystem investments</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>Investing in companies that drive GPU demand</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>Co-lead of OpenAI $110B round</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>Sequoia Capital</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>VC</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>Menlo Park, CA</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>OpenAI; Anthropic; broad AI portfolio</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>Early-stage to growth; identifying AI platform winners</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="inlineStr">
+        <is>
+          <t>Consistently backing winners across AI waves</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>Andreessen Horowitz (a16z)</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>VC</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>Menlo Park, CA</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>Broad AI portfolio: infrastructure, apps, AGI</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>AGI infrastructure thesis; AI-native application layer</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>Dedicated AI fund; prolific deal flow</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>Founders Fund (Brian Singerman)</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>VC</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>San Francisco, CA</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>OpenAI (2016), Anduril, Scale AI, Applied Intuition</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>Contrarian deep-tech bets; early conviction in frontier AI</t>
+        </is>
+      </c>
+      <c r="G35" s="2" t="inlineStr">
+        <is>
+          <t>18.3x avg returns — 3x industry average</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>Coatue Management</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>Hedge Fund / VC</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>New York, NY</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>Hugging Face, Runway, Notion, Weights &amp; Biases</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>AI-native software &amp; developer infra; AI-augmented deal sourcing</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>$70B AUM; $45M/yr on proprietary AI data infra</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>Iconiq Capital</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>Growth</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>San Francisco, CA</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>Anthropic ($13B round lead, Sep 2025)</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>Late-stage growth in proven AI platforms</t>
+        </is>
+      </c>
+      <c r="G37" s="2" t="inlineStr">
+        <is>
+          <t>Led one of the largest AI deals of 2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>Elad Gil</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>Angel / Individual</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>San Francisco, CA</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>Perplexity, Cognition, Scale AI — 36 AI deals since Jan 2024</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>High-volume seed investing; application layer focus</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t>#1 ranked AI angel investor by deal count</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>Vinod Khosla / Khosla Ventures</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>VC / Angel</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>Menlo Park, CA</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>OpenAI ($50M early, 2019); robotics, medtech, AI startups</t>
+        </is>
+      </c>
+      <c r="F39" s="2" t="inlineStr">
+        <is>
+          <t>Early conviction; patient capital through hype cycles</t>
+        </is>
+      </c>
+      <c r="G39" s="2" t="inlineStr">
+        <is>
+          <t>TIME 100 Most Influential in AI 2024</t>
+        </is>
+      </c>
+    </row>
+    <row r="40"/>
+    <row r="41">
+      <c r="A41" s="3" t="inlineStr">
+        <is>
+          <t>HOTSPOTS</t>
+        </is>
+      </c>
+      <c r="B41" s="4" t="n"/>
+      <c r="C41" s="4" t="n"/>
+      <c r="D41" s="4" t="n"/>
+      <c r="E41" s="4" t="n"/>
+      <c r="F41" s="4" t="n"/>
+      <c r="G41" s="5" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="6" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B42" s="6" t="inlineStr">
+        <is>
+          <t>City / Region</t>
+        </is>
+      </c>
+      <c r="C42" s="6" t="inlineStr">
+        <is>
+          <t>Country</t>
+        </is>
+      </c>
+      <c r="D42" s="6" t="inlineStr">
+        <is>
+          <t>AI Funding Concentration</t>
+        </is>
+      </c>
+      <c r="E42" s="6" t="inlineStr">
+        <is>
+          <t>Key Strengths</t>
+        </is>
+      </c>
+      <c r="F42" s="6" t="inlineStr">
+        <is>
+          <t>Notable Companies</t>
+        </is>
+      </c>
+      <c r="G42" s="6" t="inlineStr">
+        <is>
+          <t>Recent Developments</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>San Francisco / Silicon Valley</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>62-65% of global AI-native funding</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>Foundation models, VC density, talent pool, compute infrastructure</t>
+        </is>
+      </c>
+      <c r="F43" s="2" t="inlineStr">
+        <is>
+          <t>OpenAI, Anthropic, xAI, Scale AI, Cursor, Perplexity, NVIDIA</t>
+        </is>
+      </c>
+      <c r="G43" s="2" t="inlineStr">
+        <is>
+          <t>Epicenter of $110B OpenAI &amp; $30B Anthropic rounds</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>Seattle</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>Major North American AI center</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>Cloud infrastructure (AWS, Azure); enterprise AI; UW research</t>
+        </is>
+      </c>
+      <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t>Microsoft, Amazon/AWS, Allen Institute for AI</t>
+        </is>
+      </c>
+      <c r="G44" s="2" t="inlineStr">
+        <is>
+          <t>Microsoft AI division expansion; AWS as backbone of AI compute</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>New York</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>Major North American AI center</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>AI in finance, media, advertising; enterprise applications</t>
+        </is>
+      </c>
+      <c r="F45" s="2" t="inlineStr">
+        <is>
+          <t>Bloomberg AI, Coatue, financial services AI startups</t>
+        </is>
+      </c>
+      <c r="G45" s="2" t="inlineStr">
+        <is>
+          <t>Growing AI startup ecosystem; financial services AI acceleration</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>Toronto-Waterloo Corridor</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>50.3% AI funding concentration</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
+          <t>Pioneer research (Hinton, U of T); strong talent; affordable vs SF</t>
+        </is>
+      </c>
+      <c r="F46" s="2" t="inlineStr">
+        <is>
+          <t>Cohere, Vector Institute, U of Toronto</t>
+        </is>
+      </c>
+      <c r="G46" s="2" t="inlineStr">
+        <is>
+          <t>Growing alternative to SF for AI talent; Cohere enterprise traction</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>Austin, TX</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>Growing AI hub</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="inlineStr">
+        <is>
+          <t>xAI/Tesla AI presence; lower cost of living; tech migration from SF</t>
+        </is>
+      </c>
+      <c r="F47" s="2" t="inlineStr">
+        <is>
+          <t>xAI, Tesla AI, growing startup ecosystem</t>
+        </is>
+      </c>
+      <c r="G47" s="2" t="inlineStr">
+        <is>
+          <t>xAI HQ; emerging as secondary AI hub</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>Boston / Cambridge</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>Major AI research center</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>MIT, Harvard AI research; biotech AI; strong academic pipeline</t>
+        </is>
+      </c>
+      <c r="F48" s="2" t="inlineStr">
+        <is>
+          <t>MIT CSAIL, Harvard AI, biotech AI startups</t>
+        </is>
+      </c>
+      <c r="G48" s="2" t="inlineStr">
+        <is>
+          <t>AI-biotech convergence; strong research-to-startup pipeline</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A22:G22"/>
+    <mergeCell ref="A29:G29"/>
+    <mergeCell ref="A41:G41"/>
+    <mergeCell ref="A11:G11"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G44"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="33" customWidth="1" min="2" max="2"/>
+    <col width="50" customWidth="1" min="3" max="3"/>
+    <col width="36" customWidth="1" min="4" max="4"/>
+    <col width="50" customWidth="1" min="5" max="5"/>
+    <col width="50" customWidth="1" min="6" max="6"/>
+    <col width="50" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>LEADERS</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="n"/>
+      <c r="C1" s="4" t="n"/>
+      <c r="D1" s="4" t="n"/>
+      <c r="E1" s="4" t="n"/>
+      <c r="F1" s="4" t="n"/>
+      <c r="G1" s="5" t="n"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B2" s="6" t="inlineStr">
+        <is>
+          <t>Leader</t>
+        </is>
+      </c>
+      <c r="C2" s="6" t="inlineStr">
+        <is>
+          <t>Title / Company</t>
+        </is>
+      </c>
+      <c r="D2" s="6" t="inlineStr">
+        <is>
+          <t>HQ</t>
+        </is>
+      </c>
+      <c r="E2" s="6" t="inlineStr">
+        <is>
+          <t>Key Achievements (Past 12 Months)</t>
+        </is>
+      </c>
+      <c r="F2" s="6" t="inlineStr">
+        <is>
+          <t>Why They Stand Out</t>
+        </is>
+      </c>
+      <c r="G2" s="6" t="inlineStr">
+        <is>
+          <t>Recognition</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Arthur Mensch</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>CEO &amp; Co-Founder, Mistral AI</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Paris, France</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Grew Mistral to ~$7B+ valuation; 1.1B+ monthly queries; 6.2M active developers; 40% of EU Fortune 500 deploying/piloting</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Leading European sovereign AI champion; open-source model leadership; €50M+ government contracts</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Top EMEA CEO</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Yann LeCun</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>VP &amp; Chief AI Scientist, Meta; Founder, AMI Labs</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Paris, France</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Founded AMI Labs; raised $1B seed (Europe's largest-ever) at $3.5B valuation</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Turing Award winner; open-science AI research pioneer; bridging US tech &amp; European innovation</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>Turing Award; TIME 100 AI</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Timothée Lacroix</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>CTO &amp; Co-Founder, Mistral AI</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Paris, France</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Led technical development of Mistral models incl. Mixtral MoE architecture</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>Former Meta FAIR researcher; driving European model innovation</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>Top EMEA CTO 2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Jonas Andrulis</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>CEO &amp; Founder, Aleph Alpha</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Heidelberg, Germany</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Raised $500M Series B; built Alpha ONE (Europe's fastest commercial AI data center); ISO 27001 + EU AI Act alignment</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>Leading sovereign, compliant AI for European governments &amp; enterprise</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>German AI leader</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Demis Hassabis</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>CEO, Google DeepMind</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>London, UK</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Nobel Prize in Chemistry 2024; leads DeepMind's frontier research; AlphaFold impact continues</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>World's most decorated AI researcher; bridging scientific discovery and AI</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>Nobel Prize; TIME 100 AI</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Clem Delangue</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>CEO &amp; Co-Founder, Hugging Face</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Paris, France</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Hugging Face as the GitHub of ML; millions of models hosted; critical open-source AI infrastructure</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Democratizing AI through open-source model sharing &amp; collaboration</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>Forbes 30 Under 30 alum</t>
+        </is>
+      </c>
+    </row>
+    <row r="9"/>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>COMPANIES WITH MOST MOMENTUM</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="n"/>
+      <c r="C10" s="4" t="n"/>
+      <c r="D10" s="4" t="n"/>
+      <c r="E10" s="4" t="n"/>
+      <c r="F10" s="4" t="n"/>
+      <c r="G10" s="5" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>HQ</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t>Valuation</t>
+        </is>
+      </c>
+      <c r="E11" s="6" t="inlineStr">
+        <is>
+          <t>Revenue / Growth</t>
+        </is>
+      </c>
+      <c r="F11" s="6" t="inlineStr">
+        <is>
+          <t>Key Momentum Indicators</t>
+        </is>
+      </c>
+      <c r="G11" s="6" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Mistral AI</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Paris, France</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>~$7B+ (est.)</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>$50M+ government AI contracts; 1.1B+ monthly queries; 6.2M developers (up from 1.5M)</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>40% of Europe's Fortune 500 deploying/piloting; sovereign AI leader; avg enterprise deal $1.2M/yr</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>Foundation Model / Sovereign AI</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>AMI Labs</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Paris, France</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>$3.5B (pre-money)</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>Just founded; targeting next-gen foundation models</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>$1B seed — Europe's largest-ever; backed by NVIDIA, Bezos Expeditions, Temasek, Eric Schmidt</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>Foundation Model / Open Science</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Aleph Alpha</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Heidelberg, Germany</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>~$2B+ (est.)</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>$500M Series B; Luminous &amp; PhariaAI models</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>Alpha ONE data center (512 NVIDIA A100s); EU AI Act compliant; sovereign AI for governments</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>Sovereign AI / Enterprise</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Hugging Face</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Paris, France</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>~$4.5B</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>Millions of models hosted; critical open-source infrastructure</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>GitHub of ML; growing enterprise tier; community of millions of developers</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>AI Infrastructure / Open Source</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Stability AI</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>London, UK</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>~$1B (restructured)</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>Stable Diffusion models; restructuring under new leadership</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>Pioneered open-source image generation; expanding into video &amp; 3D</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>Generative Media / Open Source</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>DeepL</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Cologne, Germany</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>~$2B</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>AI translation leader; expanding enterprise customer base</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>Superior translation quality vs. Google Translate; strong enterprise moat</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>AI Translation / Enterprise NLP</t>
+        </is>
+      </c>
+    </row>
+    <row r="18"/>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>BIGGEST BREAKTHROUGHS</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="n"/>
+      <c r="C19" s="4" t="n"/>
+      <c r="D19" s="4" t="n"/>
+      <c r="E19" s="4" t="n"/>
+      <c r="F19" s="4" t="n"/>
+      <c r="G19" s="5" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="6" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B20" s="6" t="inlineStr">
+        <is>
+          <t>Breakthrough</t>
+        </is>
+      </c>
+      <c r="C20" s="6" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="D20" s="6" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="E20" s="6" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="F20" s="6" t="inlineStr">
+        <is>
+          <t>Impact</t>
+        </is>
+      </c>
+      <c r="G20" s="6" t="inlineStr">
+        <is>
+          <t>Technical Details</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>AMI Labs $1B Seed Round</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>AMI Labs (Yann LeCun)</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>Mar 2026</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>Europe's largest-ever seed round at $3.5B valuation for next-gen foundation models</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>Signals growing European competitiveness in frontier AI; open-science approach</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>Backed by Cathay Innovation, Bezos Expeditions, NVIDIA, Eric Schmidt, Temasek</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Mistral Sovereign AI Adoption</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>Mistral AI</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>2025-2026</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>40% of Europe's Fortune 500 deploying or piloting Mistral models; €50M+ government contracts</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>Established European sovereign AI as a viable category; EU compliance leadership</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>Open-source multilingual models; EU AI Act aligned; enterprise deals avg $1.2M/yr</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Aleph Alpha PhariaAI Stack</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>Aleph Alpha</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>Enterprise-ready generative AI stack with transparency, compliance, and data sovereignty</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>Proved sovereign AI can compete on quality; ISO 27001 + EU AI Act compliance</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>Alpha ONE: Europe's fastest commercial AI data center (512 A100s)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Demis Hassabis Nobel Prize</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>Google DeepMind (London)</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>Oct 2024</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>Nobel Prize in Chemistry for protein structure prediction (AlphaFold)</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>AI's biggest scientific validation; demonstrates AI's potential for scientific discovery</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>AlphaFold has been used by 2M+ researchers worldwide</t>
+        </is>
+      </c>
+    </row>
+    <row r="25"/>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>TOP INVESTORS</t>
+        </is>
+      </c>
+      <c r="B26" s="4" t="n"/>
+      <c r="C26" s="4" t="n"/>
+      <c r="D26" s="4" t="n"/>
+      <c r="E26" s="4" t="n"/>
+      <c r="F26" s="4" t="n"/>
+      <c r="G26" s="5" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="6" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B27" s="6" t="inlineStr">
+        <is>
+          <t>Investor / Firm</t>
+        </is>
+      </c>
+      <c r="C27" s="6" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="D27" s="6" t="inlineStr">
+        <is>
+          <t>HQ</t>
+        </is>
+      </c>
+      <c r="E27" s="6" t="inlineStr">
+        <is>
+          <t>Notable Gen AI Investments</t>
+        </is>
+      </c>
+      <c r="F27" s="6" t="inlineStr">
+        <is>
+          <t>Investment Thesis</t>
+        </is>
+      </c>
+      <c r="G27" s="6" t="inlineStr">
+        <is>
+          <t>Standout Metric</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>Bpifrance</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>State Investment Bank</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>Paris, France</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>54 AI investments; €500K-€20M tickets; broad French AI ecosystem</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>Government-backed AI development; sovereign AI support</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>Most active European AI investor by deal count</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>Cathay Innovation</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>VC</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>Paris, France</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>AMI Labs (co-led $1B seed); broad AI portfolio</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>Co-led Europe's largest-ever seed round; deep tech focus</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>€1B+ AI-focused fund</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>LocalGlobe</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>VC</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>London, UK</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>43 AI investments; early-stage focus</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>Seed to Series A; London-centric AI ecosystem development</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>2nd most active European AI VC</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>Index Ventures</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>VC</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>London / SF</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>Broad AI portfolio across Europe and US</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>Cross-Atlantic AI investing; growth-stage focus</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>Major European VC with global reach</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>Speedinvest</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>VC</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>Vienna, Austria</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>40 AI investments; €200K-€3M tickets</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>Pan-European early-stage AI; DACH region strength</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>4th most active European AI VC</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>HTGF (High-Tech Gründerfonds)</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>VC</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>Bonn, Germany</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>39 AI investments; €100K-€1M tickets</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>Deep-tech seed investing; German AI ecosystem builder</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="inlineStr">
+        <is>
+          <t>5th most active European AI VC</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>IQ Capital</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>VC</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>Cambridge / London, UK</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>39 AI investments; £500K-£10M tickets</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>Deep-tech AI and hard science; Oxbridge pipeline</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>Strong research-to-startup pipeline</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>Balderton Capital</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>VC</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>London, UK</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>Broad AI portfolio; growth-stage European AI</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>Series A-B focused; European AI scaling</t>
+        </is>
+      </c>
+      <c r="G35" s="2" t="inlineStr">
+        <is>
+          <t>Top-tier London VC</t>
+        </is>
+      </c>
+    </row>
+    <row r="36"/>
+    <row r="37">
+      <c r="A37" s="3" t="inlineStr">
+        <is>
+          <t>HOTSPOTS</t>
+        </is>
+      </c>
+      <c r="B37" s="4" t="n"/>
+      <c r="C37" s="4" t="n"/>
+      <c r="D37" s="4" t="n"/>
+      <c r="E37" s="4" t="n"/>
+      <c r="F37" s="4" t="n"/>
+      <c r="G37" s="5" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="6" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B38" s="6" t="inlineStr">
+        <is>
+          <t>City / Region</t>
+        </is>
+      </c>
+      <c r="C38" s="6" t="inlineStr">
+        <is>
+          <t>Country</t>
+        </is>
+      </c>
+      <c r="D38" s="6" t="inlineStr">
+        <is>
+          <t>AI Funding Concentration</t>
+        </is>
+      </c>
+      <c r="E38" s="6" t="inlineStr">
+        <is>
+          <t>Key Strengths</t>
+        </is>
+      </c>
+      <c r="F38" s="6" t="inlineStr">
+        <is>
+          <t>Notable Companies</t>
+        </is>
+      </c>
+      <c r="G38" s="6" t="inlineStr">
+        <is>
+          <t>Recent Developments</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>Paris</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>4.3% of global AI-native funding</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>Foundation models (Mistral, AMI Labs); strong academia (INRIA, ENS); EU sovereign AI</t>
+        </is>
+      </c>
+      <c r="F39" s="2" t="inlineStr">
+        <is>
+          <t>Mistral AI, AMI Labs, Hugging Face</t>
+        </is>
+      </c>
+      <c r="G39" s="2" t="inlineStr">
+        <is>
+          <t>AMI Labs $1B seed; Mistral in 40% EU Fortune 500; EU sovereign AI contracts</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>London</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>Major and growing AI hub</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>World-class research (DeepMind); regulatory leadership; top universities</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t>Google DeepMind, Stability AI, Faculty AI</t>
+        </is>
+      </c>
+      <c r="G40" s="2" t="inlineStr">
+        <is>
+          <t>OpenAI named London its largest research hub outside SF (Feb 2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>Zurich</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>Specialized AI hub</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>Smart city apps; fintech AI; ETH Zurich research; Google research presence</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="inlineStr">
+        <is>
+          <t>ETH Zurich, Google Brain Zurich, fintech AI startups</t>
+        </is>
+      </c>
+      <c r="G41" s="2" t="inlineStr">
+        <is>
+          <t>Leading in financial services AI; strong European research output</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>Berlin</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>Growing AI startup hub</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>Strong startup ecosystem; enterprise AI; government support</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>AI startups, enterprise SaaS with AI, research institutes</t>
+        </is>
+      </c>
+      <c r="G42" s="2" t="inlineStr">
+        <is>
+          <t>Growing pool of AI talent; lower cost than London/Paris</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>Heidelberg</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>Sovereign AI hub</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>Aleph Alpha HQ; research university strength</t>
+        </is>
+      </c>
+      <c r="F43" s="2" t="inlineStr">
+        <is>
+          <t>Aleph Alpha, Heidelberg University, EMBL</t>
+        </is>
+      </c>
+      <c r="G43" s="2" t="inlineStr">
+        <is>
+          <t>Alpha ONE data center; sovereign AI for German/EU government</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>Amsterdam-Delta</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>Netherlands</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>Emerging AI hub</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>AI in logistics, fintech, agriculture; strong tech talent</t>
+        </is>
+      </c>
+      <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t>Various AI startups; Booking.com AI; Philips AI</t>
+        </is>
+      </c>
+      <c r="G44" s="2" t="inlineStr">
+        <is>
+          <t>Growing AI investment; strategic location in Europe</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A26:G26"/>
+    <mergeCell ref="A19:G19"/>
+    <mergeCell ref="A10:G10"/>
+    <mergeCell ref="A37:G37"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G49"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="36" customWidth="1" min="2" max="2"/>
+    <col width="31" customWidth="1" min="3" max="3"/>
+    <col width="50" customWidth="1" min="4" max="4"/>
+    <col width="50" customWidth="1" min="5" max="5"/>
+    <col width="50" customWidth="1" min="6" max="6"/>
+    <col width="50" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>LEADERS</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="n"/>
+      <c r="C1" s="4" t="n"/>
+      <c r="D1" s="4" t="n"/>
+      <c r="E1" s="4" t="n"/>
+      <c r="F1" s="4" t="n"/>
+      <c r="G1" s="5" t="n"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B2" s="6" t="inlineStr">
+        <is>
+          <t>Leader</t>
+        </is>
+      </c>
+      <c r="C2" s="6" t="inlineStr">
+        <is>
+          <t>Title / Company</t>
+        </is>
+      </c>
+      <c r="D2" s="6" t="inlineStr">
+        <is>
+          <t>HQ</t>
+        </is>
+      </c>
+      <c r="E2" s="6" t="inlineStr">
+        <is>
+          <t>Key Achievements (Past 12 Months)</t>
+        </is>
+      </c>
+      <c r="F2" s="6" t="inlineStr">
+        <is>
+          <t>Why They Stand Out</t>
+        </is>
+      </c>
+      <c r="G2" s="6" t="inlineStr">
+        <is>
+          <t>Recognition</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Liang Wenfeng</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>CEO, DeepSeek</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Hangzhou, China</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>DeepSeek-V3.2 &amp; V3.2-Speciale matched/exceeded GPT-5; R1 demonstrated RL-only reasoning; all open-sourced MIT</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Frontier AI at 1/30th US cost; gold-medal results in IMO, IOI, ICPC; reshaped global AI cost economics</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Robin Li (Li Yanhong)</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>CEO, Baidu</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Beijing, China</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Leading Baidu's ERNIE Bot and enterprise AI platform in China</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>China's leading search company pivoting to AI-first; massive Chinese language data advantage</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>China AI leader</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Masayoshi Son</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>CEO, SoftBank Group</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Tokyo, Japan</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Led $40B OpenAI investment (Mar 2025); $30B follow-on (Feb 2026); cumulative $64.6B in OpenAI (~13% ownership)</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>All-in bet on AI infrastructure; largest individual AI investor globally; Stargate data center initiative</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>TIME 100 AI</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Ravi Kumar S</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>CEO, Cognizant</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Teaneck, NJ (HQ) / India ops</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Bet $1B on Gen AI; Agent Foundry for enterprise AI; Synapse to train 2M people in Gen AI</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>Driving large-scale enterprise AI transformation with major India-based workforce</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>TIME 100 AI 2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Zhang Peng</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>CEO, Zhipu AI</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Beijing, China</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>GLM-5 reached top spot among open-source models on Artificial Analysis (Feb 2026); raised prices 30% on surging demand</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>Leading China's open-source AI model race; shares rose 34%</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>China AI leader</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Yang Zhilin</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>CEO &amp; Founder, Moonshot AI</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Beijing, China</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Kimi K2 model launch (Jul 2025); briefly held top benchmarks before being surpassed</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>China's fast-moving AI startup leader; $2.5B valuation; aggressive model iteration</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>Forbes China 30 Under 30</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Pratyush Kumar</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>CEO &amp; Co-Founder, Sarvam AI</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Bengaluru, India</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>Sarvam Vision OCR at 84.3% accuracy (outperforming Gemini 3 Pro &amp; ChatGPT); Bulbul V3 TTS in 11 Indian languages</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>Building sovereign AI for Indian languages; democratizing AI for 1.4B people</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>India AI pioneer</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Ankush Sabharwal</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>CEO &amp; Founder, CoRover.ai</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>BharatGPT — India's first LLM-based Gen AI platform; 1B+ users served</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>India's homegrown Gen AI leader; conversational AI at scale</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>Top 10 global tech entrepreneur</t>
+        </is>
+      </c>
+    </row>
+    <row r="11"/>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>COMPANIES WITH MOST MOMENTUM</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="n"/>
+      <c r="C12" s="4" t="n"/>
+      <c r="D12" s="4" t="n"/>
+      <c r="E12" s="4" t="n"/>
+      <c r="F12" s="4" t="n"/>
+      <c r="G12" s="5" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="C13" s="6" t="inlineStr">
+        <is>
+          <t>HQ</t>
+        </is>
+      </c>
+      <c r="D13" s="6" t="inlineStr">
+        <is>
+          <t>Valuation</t>
+        </is>
+      </c>
+      <c r="E13" s="6" t="inlineStr">
+        <is>
+          <t>Revenue / Growth</t>
+        </is>
+      </c>
+      <c r="F13" s="6" t="inlineStr">
+        <is>
+          <t>Key Momentum Indicators</t>
+        </is>
+      </c>
+      <c r="G13" s="6" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>DeepSeek</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Hangzhou, China</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Private (self-funded)</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>Rapidly growing user base and API adoption globally</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>V3.2 matched/exceeded GPT-5 at dramatically lower cost; open-source MIT; gold-medal competition results</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>Foundation Model / Open Source</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Zhipu AI</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Beijing, China</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>~$5B+ (est.)</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>GLM-5 topped open-source benchmarks (Feb 2026); raised prices 30% on demand surge</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>Top open-source model globally; shares up 34%; intense competitive pace</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>Foundation Model / Open Source</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>ByteDance (Doubao/Seedance)</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Beijing, China</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Part of $220B+ parent</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>Seedance 2.0 video model competing with OpenAI Sora; massive user base</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>Video generation breakthrough; leveraging TikTok/Douyin distribution</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>Generative Media / Video</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Moonshot AI (Kimi)</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Beijing, China</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>$2.5B+</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>Kimi K2 model launch; aggressive model iteration cycle</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>Fast-moving Chinese AI startup; briefly held top benchmarks</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>Foundation Model / Consumer AI</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Sarvam AI</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Bengaluru, India</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>~$200M+ (est.)</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>Industry-leading OCR (84.3%); TTS in 11 Indian languages</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>Sovereign AI for India; outperforming Gemini &amp; ChatGPT on Indian language tasks</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>Sovereign AI / Indian Languages</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>CoRover.ai (BharatGPT)</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>~$100M+ (est.)</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>1B+ users served; India's first LLM-based Gen AI platform</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>Conversational AI at massive scale for Indian market</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>Conversational AI / Indian Market</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Alibaba (Qwen)</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>Hangzhou, China</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>Part of $200B+ parent</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>Qwen models; Qwen-3.5 debut expected soon</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>Leveraging Alibaba Cloud for AI distribution; open-source models</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>Foundation Model / Cloud AI</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Saltlux (LUXIA)</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>Seoul, South Korea</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>~$500M (est.)</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>LUXIA 2.5 model; virtual human video generation (Plunit Studio)</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>Korean AI leader competing with Chinese models; NLP specialist</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>Foundation Model / NLP</t>
+        </is>
+      </c>
+    </row>
+    <row r="22"/>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>BIGGEST BREAKTHROUGHS</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="n"/>
+      <c r="C23" s="4" t="n"/>
+      <c r="D23" s="4" t="n"/>
+      <c r="E23" s="4" t="n"/>
+      <c r="F23" s="4" t="n"/>
+      <c r="G23" s="5" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="6" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B24" s="6" t="inlineStr">
+        <is>
+          <t>Breakthrough</t>
+        </is>
+      </c>
+      <c r="C24" s="6" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="D24" s="6" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="E24" s="6" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="F24" s="6" t="inlineStr">
+        <is>
+          <t>Impact</t>
+        </is>
+      </c>
+      <c r="G24" s="6" t="inlineStr">
+        <is>
+          <t>Technical Details</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>DeepSeek-R1: RL-Only Reasoning</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>DeepSeek (China)</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>Jan 2025</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>First demonstration of reasoning from pure reinforcement learning without supervised fine-tuning</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>Paradigm shift; frontier AI at 1/30th US cost; open-sourced under MIT</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>R1-Zero via pure RL; R1 matches OpenAI o1; distilled 32B outperforms o1-mini</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>DeepSeek-V3.2-Speciale</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>DeepSeek (China)</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>Dec 2025</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>Open-source model matching/surpassing GPT-5; 'Thinking in Tool-Use' innovation</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>Gold-medal results IMO, IOI, ICPC, CMO; frontier model under MIT License</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>685B params, ~37B active (MoE); Sparse Attention O(L^2)→O(L); 85K+ training tasks</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>Zhipu GLM-5 Open-Source Top Rank</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>Zhipu AI (China)</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>Feb 2026</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>GLM-5 claimed #1 open-source model on Artificial Analysis benchmarking</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>Intensified China's AI model race; shares surged 34%</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>Advanced model architecture; pricing raised 30% on demand</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>ByteDance Seedance 2.0</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>ByteDance (China)</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>Feb 2026</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>Video generation model competing with OpenAI Sora; praised during testing</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>China competitive in generative video; leverages massive distribution</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>Advanced video generation; competing with Sora quality</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>Sarvam Vision OCR</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>Sarvam AI (India)</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>84.3% accuracy on OCR benchmarks — outperforming Gemini 3 Pro and ChatGPT</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>Proved Indian-built AI can beat global leaders on specific tasks</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>Specialized for Indian scripts; Bulbul V3 TTS in 11 Indian languages</t>
+        </is>
+      </c>
+    </row>
+    <row r="30"/>
+    <row r="31">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
+          <t>TOP INVESTORS</t>
+        </is>
+      </c>
+      <c r="B31" s="4" t="n"/>
+      <c r="C31" s="4" t="n"/>
+      <c r="D31" s="4" t="n"/>
+      <c r="E31" s="4" t="n"/>
+      <c r="F31" s="4" t="n"/>
+      <c r="G31" s="5" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="6" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B32" s="6" t="inlineStr">
+        <is>
+          <t>Investor / Firm</t>
+        </is>
+      </c>
+      <c r="C32" s="6" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="D32" s="6" t="inlineStr">
+        <is>
+          <t>HQ</t>
+        </is>
+      </c>
+      <c r="E32" s="6" t="inlineStr">
+        <is>
+          <t>Notable Gen AI Investments</t>
+        </is>
+      </c>
+      <c r="F32" s="6" t="inlineStr">
+        <is>
+          <t>Investment Thesis</t>
+        </is>
+      </c>
+      <c r="G32" s="6" t="inlineStr">
+        <is>
+          <t>Standout Metric</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>SoftBank Group / Vision Fund</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>VC / Growth</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>Tokyo, Japan</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>OpenAI ($64.6B cumulative ~13% ownership); xAI; Stargate initiative</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>All-in bet on AI infrastructure; largest individual AI investor globally</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="inlineStr">
+        <is>
+          <t>Led two largest private funding rounds in history</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>Temasek</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>Sovereign Wealth Fund</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>Singapore</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>AMI Labs; Upscale AI ($200M round); bullish on China AI (B2B focus)</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>AI infrastructure and B2B applications; True Light Capital for China innovation</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>Invested across US, EU, and Asian AI ecosystems</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>Premji Invest</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>Family Office</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>Bengaluru, India</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>Upscale AI ($200M Series A); Indian AI ecosystem investments</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>Indian AI infrastructure and enterprise applications</t>
+        </is>
+      </c>
+      <c r="G35" s="2" t="inlineStr">
+        <is>
+          <t>Co-investor in major Indian AI rounds</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>Alibaba Group</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>Strategic / Corporate</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>Hangzhou, China</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>Qwen models; Alibaba Cloud AI; internal AI investments</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>Cloud AI infrastructure; open-source model ecosystem</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>Major corporate AI investor in China</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>Tencent</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>Strategic / Corporate</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>Shenzhen, China</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>AI Lab investments; gaming AI; WeChat AI integrations</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>Consumer AI via social/gaming platforms; enterprise AI emerging</t>
+        </is>
+      </c>
+      <c r="G37" s="2" t="inlineStr">
+        <is>
+          <t>One of China's largest AI corporate investors</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>Shorooq Partners</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>VC</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>UAE / Middle East</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>AMI Labs ($1B seed participant); MENA AI ecosystem</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>Bridging Middle East capital with global AI ventures</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t>Expanding into frontier AI investments globally</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>Xora Innovation (Temasek-backed)</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>VC</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>Singapore</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>Upscale AI ($200M Series A); Southeast Asian AI ecosystem</t>
+        </is>
+      </c>
+      <c r="F39" s="2" t="inlineStr">
+        <is>
+          <t>AI infrastructure and B2B applications in Asia</t>
+        </is>
+      </c>
+      <c r="G39" s="2" t="inlineStr">
+        <is>
+          <t>Active participant in large Asian AI rounds</t>
+        </is>
+      </c>
+    </row>
+    <row r="40"/>
+    <row r="41">
+      <c r="A41" s="3" t="inlineStr">
+        <is>
+          <t>HOTSPOTS</t>
+        </is>
+      </c>
+      <c r="B41" s="4" t="n"/>
+      <c r="C41" s="4" t="n"/>
+      <c r="D41" s="4" t="n"/>
+      <c r="E41" s="4" t="n"/>
+      <c r="F41" s="4" t="n"/>
+      <c r="G41" s="5" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="6" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B42" s="6" t="inlineStr">
+        <is>
+          <t>City / Region</t>
+        </is>
+      </c>
+      <c r="C42" s="6" t="inlineStr">
+        <is>
+          <t>Country</t>
+        </is>
+      </c>
+      <c r="D42" s="6" t="inlineStr">
+        <is>
+          <t>AI Funding Concentration</t>
+        </is>
+      </c>
+      <c r="E42" s="6" t="inlineStr">
+        <is>
+          <t>Key Strengths</t>
+        </is>
+      </c>
+      <c r="F42" s="6" t="inlineStr">
+        <is>
+          <t>Notable Companies</t>
+        </is>
+      </c>
+      <c r="G42" s="6" t="inlineStr">
+        <is>
+          <t>Recent Developments</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>Beijing</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>66.2% of local startup funding goes to AI — highest globally</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>Foundation models at 1/30th US cost; massive government support; large talent pool</t>
+        </is>
+      </c>
+      <c r="F43" s="2" t="inlineStr">
+        <is>
+          <t>DeepSeek, Baidu, ByteDance, Zhipu AI, Moonshot AI</t>
+        </is>
+      </c>
+      <c r="G43" s="2" t="inlineStr">
+        <is>
+          <t>DeepSeek breakthroughs reshaped global AI cost economics</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>Shanghai / Greater Bay Area</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>Emerging AI powerhouse</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>Hardware manufacturing ecosystem; application-layer AI; massive consumer market</t>
+        </is>
+      </c>
+      <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t>Alibaba AI, Tencent AI Lab, semiconductor ecosystem</t>
+        </is>
+      </c>
+      <c r="G44" s="2" t="inlineStr">
+        <is>
+          <t>Growing AI applications; connection to hardware supply chain (Shenzhen)</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>Singapore</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>Singapore</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>Growing AI investment hub</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>World's best AI readiness; government-wide implementation; governance leadership</t>
+        </is>
+      </c>
+      <c r="F45" s="2" t="inlineStr">
+        <is>
+          <t>AI Singapore, Temasek AI investments, SEA hub</t>
+        </is>
+      </c>
+      <c r="G45" s="2" t="inlineStr">
+        <is>
+          <t>Leading AI governance frameworks; attracting global AI companies</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>Bengaluru</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>India's #1 AI hub</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
+          <t>Massive talent pool; growing startup ecosystem; enterprise AI services</t>
+        </is>
+      </c>
+      <c r="F46" s="2" t="inlineStr">
+        <is>
+          <t>Sarvam AI, CoRover.ai, Infosys AI, Wipro AI</t>
+        </is>
+      </c>
+      <c r="G46" s="2" t="inlineStr">
+        <is>
+          <t>Indian sovereign AI movement; language-specific AI innovation</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>Tokyo</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t>Japan</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>Rising AI investment center</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="inlineStr">
+        <is>
+          <t>Robotics AI; industrial automation; SoftBank HQ; strong R&amp;D culture</t>
+        </is>
+      </c>
+      <c r="F47" s="2" t="inlineStr">
+        <is>
+          <t>SoftBank, NEC, Preferred Networks, Sakana AI</t>
+        </is>
+      </c>
+      <c r="G47" s="2" t="inlineStr">
+        <is>
+          <t>SoftBank's massive AI investment strategy; growing AI startup scene</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>Seoul</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>South Korea</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>Specialized AI hub</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>NLP and conversational AI; Samsung/LG AI divisions; gaming AI</t>
+        </is>
+      </c>
+      <c r="F48" s="2" t="inlineStr">
+        <is>
+          <t>Saltlux, Samsung AI, Naver, Kakao</t>
+        </is>
+      </c>
+      <c r="G48" s="2" t="inlineStr">
+        <is>
+          <t>LUXIA 2.5 model; growing Korean AI ecosystem</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>Hangzhou</t>
+        </is>
+      </c>
+      <c r="C49" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="inlineStr">
+        <is>
+          <t>DeepSeek's home city</t>
+        </is>
+      </c>
+      <c r="E49" s="2" t="inlineStr">
+        <is>
+          <t>Alibaba ecosystem; DeepSeek research lab; e-commerce AI</t>
+        </is>
+      </c>
+      <c r="F49" s="2" t="inlineStr">
+        <is>
+          <t>DeepSeek, Alibaba, e-commerce AI startups</t>
+        </is>
+      </c>
+      <c r="G49" s="2" t="inlineStr">
+        <is>
+          <t>DeepSeek's breakthroughs put Hangzhou on the global AI map</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A31:G31"/>
+    <mergeCell ref="A12:G12"/>
+    <mergeCell ref="A41:G41"/>
+    <mergeCell ref="A23:G23"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add Agentic AI & OpenClaw ecosystem tab (Tab 10)
New tab covers the full agentic AI landscape with 4 sections:

1. OpenClaw & Open-Source Agent Runtimes (5 entries):
   OpenClaw (234K stars, 1.5M agents), LangChain/LangGraph,
   CrewAI, AutoGen, n8n

2. Venture-Backed Agentic AI Startups (10 entries):
   Cognition/Devin ($10.2B), Temporal ($5B), Gumloop, Adept,
   Simular, Relevance AI, Daytona, Sapiom, Lindy AI, Genspark Claw

3. Big Tech Agentic AI Products (4 entries):
   OpenAI Operator, Claude Computer Use/Code, Google Mariner,
   Microsoft Copilot Agents

4. Market Landscape Summary: category leaders and trends

Co-authored-by: ms4674 <ms4674@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/generative_ai_market_insights.xlsx
+++ b/generative_ai_market_insights.xlsx
@@ -16,6 +16,7 @@
     <sheet name="Americas" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="Europe" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="Asia" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Agentic AI &amp; OpenClaw" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -867,6 +868,1199 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H35"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="44" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="39" customWidth="1" min="3" max="3"/>
+    <col width="50" customWidth="1" min="4" max="4"/>
+    <col width="50" customWidth="1" min="5" max="5"/>
+    <col width="50" customWidth="1" min="6" max="6"/>
+    <col width="50" customWidth="1" min="7" max="7"/>
+    <col width="50" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>OPENCLAW &amp; OPEN-SOURCE AI AGENT RUNTIMES</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="n"/>
+      <c r="C1" s="4" t="n"/>
+      <c r="D1" s="4" t="n"/>
+      <c r="E1" s="4" t="n"/>
+      <c r="F1" s="4" t="n"/>
+      <c r="G1" s="4" t="n"/>
+      <c r="H1" s="5" t="n"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B2" s="6" t="inlineStr">
+        <is>
+          <t>Project / Company</t>
+        </is>
+      </c>
+      <c r="C2" s="6" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="D2" s="6" t="inlineStr">
+        <is>
+          <t>HQ / Origin</t>
+        </is>
+      </c>
+      <c r="E2" s="6" t="inlineStr">
+        <is>
+          <t>GitHub Stars / Adoption</t>
+        </is>
+      </c>
+      <c r="F2" s="6" t="inlineStr">
+        <is>
+          <t>Key Capabilities</t>
+        </is>
+      </c>
+      <c r="G2" s="6" t="inlineStr">
+        <is>
+          <t>Funding / Business Model</t>
+        </is>
+      </c>
+      <c r="H2" s="6" t="inlineStr">
+        <is>
+          <t>Status (Mar 2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>OpenClaw</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Open-Source AI Agent Runtime</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Austria (founder); now OpenAI-affiliated</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>234K+ GitHub stars; 1.5M+ agents running; #1 GitHub repo (early 2026)</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Autonomous agent execution via LLMs (GPT, Claude); shell commands, file management, email, messaging (WhatsApp/Slack/Telegram/Discord); web browsing; persistent memory; heartbeat daemon for continuous operation; 7,400+ MCP skills</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Free &amp; open-source (MIT); LLM API costs ~$10-50/mo; founder Peter Steinberger joined OpenAI Feb 2026; project transitioned to independent foundation</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>Fastest-growing open-source AI project; security vulnerability CVE-2026-25253 patched; foundation governance established</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>LangChain / LangGraph</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Open-Source Agent Framework</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>San Francisco, CA (USA)</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>90K+ GitHub stars (LangChain); wide enterprise adoption</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Agent orchestration with explicit state management; human-in-the-loop controls; 1,000+ integrations; durable runtime; streaming &amp; memory persistence; best for complex pipelines with branching logic</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>VC-backed (Sequoia-led $25M Series A); LangSmith commercial SaaS for observability/monitoring</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>Preferred framework for production-grade agent complexity; Daytona ($24M) partnership</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>CrewAI</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Open-Source Multi-Agent Framework</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>100K+ certified developers; fast-growing community</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>Autonomous collaborative agents (Crews) + event-driven production workflows (Flows); lightweight Python framework; simple high-level abstractions for multi-agent teams</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>VC-backed; CrewAI Enterprise for commercial use</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>Standard for enterprise AI team automation; simpler alternative to LangGraph</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>AutoGen</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Open-Source Agent Framework</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Microsoft Research</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Strong adoption in research &amp; enterprise</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>Chat-based multi-agent conversations; best for two-agent dialogue patterns; Microsoft ecosystem integration</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>Microsoft-backed open-source project</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>Solid for chat-based agent patterns; less ideal for complex branching pipelines</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>n8n</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Open-Source Workflow Automation</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Berlin, Germany</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>60K+ GitHub stars; 1,700+ community templates</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>Visual node-based workflow builder; 400+ pre-built integrations; deterministic trigger-based pipelines; complements OpenClaw for structured workflows</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>Free self-host; cloud from €24/mo; VC-backed</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>Complementary to OpenClaw; used together for hybrid AI+deterministic automation</t>
+        </is>
+      </c>
+    </row>
+    <row r="8"/>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>AGENTIC AI STARTUPS (VENTURE-BACKED)</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="n"/>
+      <c r="C9" s="4" t="n"/>
+      <c r="D9" s="4" t="n"/>
+      <c r="E9" s="4" t="n"/>
+      <c r="F9" s="4" t="n"/>
+      <c r="G9" s="4" t="n"/>
+      <c r="H9" s="5" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>Focus Area</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="inlineStr">
+        <is>
+          <t>HQ</t>
+        </is>
+      </c>
+      <c r="E10" s="6" t="inlineStr">
+        <is>
+          <t>Valuation / Funding</t>
+        </is>
+      </c>
+      <c r="F10" s="6" t="inlineStr">
+        <is>
+          <t>Key Product / Capability</t>
+        </is>
+      </c>
+      <c r="G10" s="6" t="inlineStr">
+        <is>
+          <t>Notable Customers / Metrics</t>
+        </is>
+      </c>
+      <c r="H10" s="6" t="inlineStr">
+        <is>
+          <t>Momentum</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Cognition (Devin)</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Autonomous Coding Agent</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>San Francisco, CA</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>$10.2B valuation; $400M raised (Sep 2025, Founders Fund-led)</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>Devin: autonomous AI software engineer that plans, codes, debugs, and deploys; acquired Windsurf IDE (Jul 2025)</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>Goldman Sachs, Citi, Dell, Cisco, Ramp, Palantir, Nubank; $73M ARR (Jun 2025, up from $1M in Sep 2024)</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>140x ARR multiple; net burn under $20M since founding; combined ARR grew 30%+ in 7 weeks post-Windsurf acquisition</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Temporal</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Durable Execution for AI Agents</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>San Francisco, CA</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>$5B valuation; $300M Series D (Feb 2026, a16z-led)</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>Durable execution infrastructure for long-running AI agents; ensures reliability and fault tolerance at production scale</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>20M+ monthly installs; 380% YoY revenue growth; 350% increase in weekly active usage</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>Critical infrastructure layer for production agentic AI; addressing reliability bottleneck</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Gumloop</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>No-Code AI Agent Builder</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>San Francisco, CA</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>$50M Series B (Benchmark-led); Y Combinator, First Round, Shopify Ventures</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>Platform enabling non-technical employees to build AI agents and automations</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>Shopify, Ramp, Instacart</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>Democratizing agent creation; enterprise adoption growing</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Adept</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Enterprise Agentic AI</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>San Francisco, CA</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>~$1B+ valuation</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>Enterprise agents that execute complex workflows across websites and software; proprietary models trained on web UI data</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>Enterprise customers across multiple verticals</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>Pioneered 'action model' approach; focused on workforce automation</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Simular</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>OS-Level Computer Use Agent</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>$21.5M Series A (Felicis-led)</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>Neuro-symbolic agents that control Mac/PC at OS level (mouse, keyboard, apps); not just browser-based</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>Mac 1.0 released; Windows version via Microsoft Windows 365 for Agents program</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>Going beyond browser to full OS control; Microsoft partnership</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Relevance AI</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>AI Agent Operating System</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Sydney, Australia</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>$24M Series B (May 2025)</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>Visual multi-agent system builder (Workforce); text-to-agent generator; enables non-technical users to build agents</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>40,000 AI agents created on platform (Jan 2025)</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>Bridging technical and non-technical agent creation</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Daytona</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Agent Compute Infrastructure</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>USA / Europe</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>$24M Series A (Feb 2026)</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>Programmatic, composable computers for AI agents that launch in milliseconds</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>LangChain, Turing, Writer, SambaNova; $1M FRR in &lt;3 months, doubled in 6 weeks</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>Solving the 'where do agents run?' problem; rapid revenue growth</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Sapiom</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Agent Financial Infrastructure</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>$15M Seed (Accel-led)</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>Financial infrastructure enabling agents to pay, authenticate, and audit their own API/cloud usage autonomously</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>Early-stage; solving agent payment and identity</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>Novel category: financial autonomy for AI agents</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Lindy AI</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Personal AI Assistant / Phone Agent</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>San Francisco, CA</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>VC-backed (undisclosed)</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>AI assistant for scheduling, email, meeting summaries; Gaia: fastest AI phone agent (&lt;500ms response)</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>Growing consumer and business user base</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>Competing in personal AI assistant space; phone agent innovation</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Genspark Claw</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>Secure Cloud AI Agent</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>Part of Genspark (VC-backed)</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>Cloud-based alternative to OpenClaw addressing enterprise security and setup complexity</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>Targeting enterprises wary of self-hosted agent security risks</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>Launched Mar 2026 as direct response to OpenClaw security concerns</t>
+        </is>
+      </c>
+    </row>
+    <row r="21"/>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>BIG TECH AGENTIC AI PRODUCTS</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="n"/>
+      <c r="C22" s="4" t="n"/>
+      <c r="D22" s="4" t="n"/>
+      <c r="E22" s="4" t="n"/>
+      <c r="F22" s="4" t="n"/>
+      <c r="G22" s="4" t="n"/>
+      <c r="H22" s="5" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="6" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B23" s="6" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="C23" s="6" t="inlineStr">
+        <is>
+          <t>Product / Initiative</t>
+        </is>
+      </c>
+      <c r="D23" s="6" t="inlineStr">
+        <is>
+          <t>Launch Date</t>
+        </is>
+      </c>
+      <c r="E23" s="6" t="inlineStr">
+        <is>
+          <t>Key Capability</t>
+        </is>
+      </c>
+      <c r="F23" s="6" t="inlineStr">
+        <is>
+          <t>Target Market</t>
+        </is>
+      </c>
+      <c r="G23" s="6" t="inlineStr">
+        <is>
+          <t>How It Compares to OpenClaw</t>
+        </is>
+      </c>
+      <c r="H23" s="6" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>GPT-5.4 Computer Use / Operator</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>Mar 2026</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>Native computer-use capabilities; autonomous agent workflows; keyboard/mouse commands across applications</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>Enterprise &amp; consumer</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>Proprietary; cloud-based; integrated into ChatGPT; less customizable than OpenClaw but more polished</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>Just launched; acquired OpenClaw founder Peter Steinberger</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>Anthropic</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>Claude Computer Use / Claude Code</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>2025-2026</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>Claude can interact with computer interfaces; Claude Code autonomous coding ($2.5B+ run-rate); 4% of GitHub public commits</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>Enterprise developers</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>API-based; enterprise-focused; Claude Code is biggest revenue-generating agent product</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>Claude Code is #1 revenue-generating AI agent product globally</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>Google</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>Gemini Agents / Project Mariner</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>2025-2026</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>Gemini 3.1 Pro agentic workflows; browser/computer use capabilities</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>Enterprise &amp; consumer</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>Cloud-based; integrated into Google ecosystem; Workspace, Search, Chrome</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>Expanding agentic capabilities across Google product suite</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>Microsoft</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>Copilot Agents / AutoGen</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>2025-2026</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>Microsoft 365 Copilot agents; AutoGen framework; Windows 365 for Agents</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>Enterprise (M365 ecosystem)</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>Deep enterprise integration; combines AutoGen open-source with proprietary Copilot</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t>Largest enterprise agent deployment via M365 Copilot</t>
+        </is>
+      </c>
+    </row>
+    <row r="28"/>
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>AGENTIC AI MARKET LANDSCAPE SUMMARY</t>
+        </is>
+      </c>
+      <c r="B29" s="4" t="n"/>
+      <c r="C29" s="4" t="n"/>
+      <c r="D29" s="4" t="n"/>
+      <c r="E29" s="4" t="n"/>
+      <c r="F29" s="4" t="n"/>
+      <c r="G29" s="4" t="n"/>
+      <c r="H29" s="5" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="6" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="B30" s="6" t="inlineStr">
+        <is>
+          <t>Leader</t>
+        </is>
+      </c>
+      <c r="C30" s="6" t="inlineStr">
+        <is>
+          <t>Runner-Up</t>
+        </is>
+      </c>
+      <c r="D30" s="6" t="inlineStr">
+        <is>
+          <t>Key Metric</t>
+        </is>
+      </c>
+      <c r="E30" s="6" t="inlineStr">
+        <is>
+          <t>Trend</t>
+        </is>
+      </c>
+      <c r="F30" s="6" t="inlineStr"/>
+      <c r="G30" s="6" t="inlineStr"/>
+      <c r="H30" s="6" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>Open-Source Agent Runtime</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>OpenClaw</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>LangChain / LangGraph</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>234K GitHub stars; 1.5M+ agents running</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>Open-source agentic AI is the fastest-growing category; security &amp; governance are top concerns</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr"/>
+      <c r="G31" s="2" t="inlineStr"/>
+      <c r="H31" s="2" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>Venture-Backed Agent Startup</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>Cognition (Devin)</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>Temporal</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>Cognition: $10.2B at $73M ARR; Temporal: $5B at 380% rev growth</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>Autonomous coding and durable execution are the two hottest agentic sub-categories</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr"/>
+      <c r="G32" s="2" t="inlineStr"/>
+      <c r="H32" s="2" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>Enterprise Agent Platform</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>Microsoft Copilot Agents</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>Anthropic Claude Code</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>Copilot: largest enterprise deployment; Claude Code: $2.5B+ run-rate</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>Enterprise agentic AI is moving from pilot to production across Fortune 500</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr"/>
+      <c r="G33" s="2" t="inlineStr"/>
+      <c r="H33" s="2" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>Agent Infrastructure</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>Temporal (durable execution)</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>Daytona (compute)</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>Temporal: $300M raise; Daytona: $1M FRR in 3 months</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>Infrastructure for where and how agents run is an emerging critical layer</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr"/>
+      <c r="G34" s="2" t="inlineStr"/>
+      <c r="H34" s="2" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>Fastest-Growing Category</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>AI Coding Agents</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>AI Personal Assistants</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>Devin $1M→$73M ARR in 9 months; Cursor $2B ARR in 18 months</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>Developer tools are the highest-velocity segment of the agentic AI market</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="inlineStr"/>
+      <c r="G35" s="2" t="inlineStr"/>
+      <c r="H35" s="2" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="A9:H9"/>
+    <mergeCell ref="A29:H29"/>
+    <mergeCell ref="A22:H22"/>
+    <mergeCell ref="A1:H1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Add AI Memory ecosystem tab (Tab 11)
New tab covers the full AI memory landscape with 4 sections:

1. Dedicated AI Memory Platforms (7 entries):
   Mem0 ($24M, AWS partnership, 186M API calls/quarter),
   Zep (knowledge graph, 98% cost reduction),
   Letta/MemGPT ($10M, Berkeley spinout),
   OMEGA (#1 LongMemEval at 95.4%),
   ReMemora, Mnexium, ContextStream

2. Vector Databases - Memory Infrastructure Layer (4 entries):
   Pinecone ($750M, a16z), Weaviate ($200-500M+),
   Chroma, SochDB

3. Big Tech AI Memory Initiatives (5 entries):
   Google Always On Memory Agent (ditching vector DBs),
   OpenAI ChatGPT Memory, Anthropic Claude Memory,
   Tabnine Enterprise Context Engine, Memori Labs

4. Market Landscape Summary:
   Best-funded: Mem0; highest benchmark: OMEGA;
   biggest paradigm shift: LLM-native memory replacing vector DBs

Co-authored-by: ms4674 <ms4674@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/generative_ai_market_insights.xlsx
+++ b/generative_ai_market_insights.xlsx
@@ -17,6 +17,7 @@
     <sheet name="Europe" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="Asia" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="Agentic AI &amp; OpenClaw" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="AI Memory" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -2061,6 +2062,1103 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H33"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="50" customWidth="1" min="1" max="1"/>
+    <col width="33" customWidth="1" min="2" max="2"/>
+    <col width="41" customWidth="1" min="3" max="3"/>
+    <col width="50" customWidth="1" min="4" max="4"/>
+    <col width="50" customWidth="1" min="5" max="5"/>
+    <col width="50" customWidth="1" min="6" max="6"/>
+    <col width="50" customWidth="1" min="7" max="7"/>
+    <col width="50" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>DEDICATED AI MEMORY PLATFORMS</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="n"/>
+      <c r="C1" s="4" t="n"/>
+      <c r="D1" s="4" t="n"/>
+      <c r="E1" s="4" t="n"/>
+      <c r="F1" s="4" t="n"/>
+      <c r="G1" s="4" t="n"/>
+      <c r="H1" s="5" t="n"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B2" s="6" t="inlineStr">
+        <is>
+          <t>Company / Project</t>
+        </is>
+      </c>
+      <c r="C2" s="6" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="D2" s="6" t="inlineStr">
+        <is>
+          <t>HQ / Origin</t>
+        </is>
+      </c>
+      <c r="E2" s="6" t="inlineStr">
+        <is>
+          <t>Funding / Valuation</t>
+        </is>
+      </c>
+      <c r="F2" s="6" t="inlineStr">
+        <is>
+          <t>Core Technology</t>
+        </is>
+      </c>
+      <c r="G2" s="6" t="inlineStr">
+        <is>
+          <t>Key Metrics / Traction</t>
+        </is>
+      </c>
+      <c r="H2" s="6" t="inlineStr">
+        <is>
+          <t>Differentiator</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Mem0</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>AI Memory Layer (Cloud + Self-Host)</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>San Francisco, CA (YC S24)</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>$24M (Seed + Series A, Oct 2025); Basis Set Ventures-led; backed by Y Combinator, Peak XV, GitHub Fund</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Production-ready memory infrastructure for AI agents; integrates in 3 lines of code; graph relationships in paid tier ($249/mo); exclusive memory provider for AWS Agent SDK</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>41K+ GitHub stars; 14M+ Python downloads; API calls grew from 35M (Q1 2025) to 186M (Q3 2025) — ~30% MoM growth; 80K+ developers on managed cloud</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>Best-funded dedicated memory startup; production focus; AWS partnership; strong angel backing (Dharmesh Shah, Scott Belsky, Datadog CEO, ex-GitHub CEO)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Zep AI</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Agent Memory Layer (Knowledge Graph)</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>San Francisco, CA (YC W24)</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>~$2.3-3.3M total (pre-seed via YC W24); $1M revenue by Jun 2024</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Temporal knowledge graph that auto-constructs from user interactions; Neo4j-backed; semantic + episodic + procedural memory types</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>94.8% DMR benchmark accuracy (outperforms MemGPT); 18.5% accuracy improvement on LongMemEval; 98% cost reduction vs full-context; 90% latency reduction</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>Research-backed performance leadership; named CB Insights 'Outperformer'; knowledge graph approach captures temporal relationships</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Letta (formerly MemGPT)</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Stateful Agent Framework</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>UC Berkeley spinout, San Francisco, CA</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>$10M Seed (Sep 2024); Felicis Ventures-led; angels incl. Jeff Dean (Google DeepMind), Clem Delangue (Hugging Face)</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>Stateful memory enabling agents to retain info across sessions; MemGPT architecture; Agent Development Environment (ADE) for debugging memory; Context Repositories (git-based memory for coding agents); Conversations API</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>Open-source community-driven; Desktop UI + CLI; model-agnostic; Letta Code terminal agent</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>Academic pedigree (Berkeley); open-source community-first approach; strongest developer tooling for inspecting/editing agent memory</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>OMEGA</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Open-Source Local Memory System</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Open Source</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Free &amp; open-source (Apache-2.0); no external funding</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>Local-first persistent memory for AI coding agents; SQLite + AES-256 encryption; semantic search via ONNX embeddings (bge-small-en-v1.5); 12 MCP tools for Claude Code/Cursor/Windsurf; intelligent forgetting with contradiction detection</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>#1 on LongMemEval benchmark: 95.4% (500 questions); production-ready v1.2.0; 36 GitHub stars</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>Highest benchmark score; fully local (no cloud dependency); zero API keys needed; privacy-first; designed specifically for AI coding agents</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>ReMemora</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Persistent Memory Infrastructure</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>USA (early-stage)</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Early-stage (undisclosed)</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>Captures and organizes insights in real-time for human-AI teams; classified memory storage; designed for autonomous agent collaboration</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>Early-stage; positioning for human-AI teaming use case</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>Unique focus on human-AI team memory — not just agent memory</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Mnexium</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Persistent Memory for LLMs</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>USA (early-stage)</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Early-stage (undisclosed)</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Provider-agnostic persistent memory (works with OpenAI, Claude, Gemini); chat history, agent state, records management, observability; 2-line integration</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>Early-stage; developer-focused</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>Simplest integration (2 lines); provider-agnostic design</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>ContextStream</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Persistent Memory for Coding Tools</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>USA (early-stage)</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>Early-stage (undisclosed)</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>Persistent memory with semantic code search for AI coding tools; deduplication and progressive compression to reduce token costs</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>Early-stage; targeting developer tools market</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>Specialized for code context; token cost optimization via compression</t>
+        </is>
+      </c>
+    </row>
+    <row r="10"/>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>VECTOR DATABASES (MEMORY INFRASTRUCTURE LAYER)</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="n"/>
+      <c r="C11" s="4" t="n"/>
+      <c r="D11" s="4" t="n"/>
+      <c r="E11" s="4" t="n"/>
+      <c r="F11" s="4" t="n"/>
+      <c r="G11" s="4" t="n"/>
+      <c r="H11" s="5" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="D12" s="6" t="inlineStr">
+        <is>
+          <t>HQ</t>
+        </is>
+      </c>
+      <c r="E12" s="6" t="inlineStr">
+        <is>
+          <t>Funding / Valuation</t>
+        </is>
+      </c>
+      <c r="F12" s="6" t="inlineStr">
+        <is>
+          <t>Core Technology</t>
+        </is>
+      </c>
+      <c r="G12" s="6" t="inlineStr">
+        <is>
+          <t>Key Metrics</t>
+        </is>
+      </c>
+      <c r="H12" s="6" t="inlineStr">
+        <is>
+          <t>Role in AI Memory</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Pinecone</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Managed Vector Database</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>San Francisco, CA</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>$138M total; $100M Series B (Apr 2023, a16z-led); $750M valuation</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>Serverless vector database; sub-33ms p99 latency at scale; Dedicated Read Nodes (Dec 2025); BYOC for enterprise; Pinecone Assistant with Claude integration</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>128 employees; critical infrastructure for RAG and AI memory pipelines</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>Most widely adopted managed vector DB; foundational layer for Mem0, Zep, and other memory platforms</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Weaviate</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Open-Source Vector Database</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Amsterdam, Netherlands</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>$50M Series B (Apr 2023, Index Ventures); $200M-$500M+ valuation</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>AI-native vector search; hybrid search (vector + keyword); AI Agents for autonomous DB operations; self-hosted + cloud; v1.35 (Dec 2025) with Object TTL and zstd compression</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>99-100+ employees; growing enterprise adoption</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>Open-source alternative to Pinecone; strong European presence; self-hosted option for data sovereignty</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Chroma</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Open-Source Embedding Database</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>San Francisco, CA</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>~$18M raised; ~$75M+ valuation (est.)</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>Developer-friendly embedding database; 20ms p50 latency; full-text + vector hybrid search; now GA cloud platform</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>Large open-source community; lowest barrier to entry</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>Most developer-friendly vector DB; popular for prototyping and small-to-mid-scale AI memory</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>SochDB</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>LLM-Native Database</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Early-stage</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>Early-stage (undisclosed)</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>Combined vector search + SQL + token-aware context budgeting in single embedded system; replaces separate vector DB + relational DB + prompt packing stacks</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>Early-stage; novel architecture</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>Next-gen: purpose-built for LLM memory, not retrofitted from vector search</t>
+        </is>
+      </c>
+    </row>
+    <row r="17"/>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>BIG TECH AI MEMORY INITIATIVES</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="n"/>
+      <c r="C18" s="4" t="n"/>
+      <c r="D18" s="4" t="n"/>
+      <c r="E18" s="4" t="n"/>
+      <c r="F18" s="4" t="n"/>
+      <c r="G18" s="4" t="n"/>
+      <c r="H18" s="5" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="6" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B19" s="6" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="C19" s="6" t="inlineStr">
+        <is>
+          <t>Product / Initiative</t>
+        </is>
+      </c>
+      <c r="D19" s="6" t="inlineStr">
+        <is>
+          <t>Launch</t>
+        </is>
+      </c>
+      <c r="E19" s="6" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="F19" s="6" t="inlineStr">
+        <is>
+          <t>Approach</t>
+        </is>
+      </c>
+      <c r="G19" s="6" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="H19" s="6" t="inlineStr">
+        <is>
+          <t>Significance</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Google</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>Always On Memory Agent (open-sourced)</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>Mar 2026</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>Open-source persistent memory agent built with Google Agent Development Kit + Gemini 3.1 Flash-Lite</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>Ditches vector databases entirely; uses LLM-driven structured memory stored in SQLite</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>Open-sourced; community adoption growing</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>Signals potential shift away from vector DBs toward LLM-native memory management</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>ChatGPT Memory / Custom Instructions</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>2024-2026</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>Persistent memory across ChatGPT conversations; remembers user preferences, facts, and context</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>Proprietary cloud-based memory integrated into ChatGPT consumer and enterprise products</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>Rolled out to all ChatGPT users; continuously improving</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>Largest-scale deployment of persistent AI memory (800-900M weekly users)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Anthropic</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>Claude Project Knowledge / Memory</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>2025-2026</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>Project-level context and memory for Claude; persistent knowledge across conversations within projects</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>Cloud-based; tied to Claude Projects feature; complements Claude Code's session persistence</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>Active development; growing enterprise adoption</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>Enterprise-grade memory for business workflows</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Tabnine</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>Enterprise Context Engine</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>Feb 2026</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>Continuously evolving model of organizational software systems, docs, and engineering practices</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>Not RAG-based; builds structural understanding of codebases; supports air-gapped environments</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>Launched; targeting enterprise development teams</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>Enterprise code memory that understands system architecture, not just text</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Memori Labs</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>Enterprise Memory Fabric</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>2025-2026</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>Classified memory storage (facts, preferences, rules, summaries) for enterprise AI</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>Tokenless recall; targeted context retrieval; claims 98% cost reduction</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>Early-stage; enterprise-focused</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>Enterprise-specific memory optimization; cost reduction focus</t>
+        </is>
+      </c>
+    </row>
+    <row r="25"/>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>AI MEMORY MARKET LANDSCAPE SUMMARY</t>
+        </is>
+      </c>
+      <c r="B26" s="4" t="n"/>
+      <c r="C26" s="4" t="n"/>
+      <c r="D26" s="4" t="n"/>
+      <c r="E26" s="4" t="n"/>
+      <c r="F26" s="4" t="n"/>
+      <c r="G26" s="4" t="n"/>
+      <c r="H26" s="5" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="6" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="B27" s="6" t="inlineStr">
+        <is>
+          <t>Leader</t>
+        </is>
+      </c>
+      <c r="C27" s="6" t="inlineStr">
+        <is>
+          <t>Runner-Up</t>
+        </is>
+      </c>
+      <c r="D27" s="6" t="inlineStr">
+        <is>
+          <t>Key Metric</t>
+        </is>
+      </c>
+      <c r="E27" s="6" t="inlineStr">
+        <is>
+          <t>Trend</t>
+        </is>
+      </c>
+      <c r="F27" s="6" t="inlineStr"/>
+      <c r="G27" s="6" t="inlineStr"/>
+      <c r="H27" s="6" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>Best-Funded Memory Startup</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>Mem0 ($24M)</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>Letta ($10M)</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>Mem0: 186M API calls/quarter, 80K developers, AWS partnership</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>Dedicated AI memory is emerging as a distinct infrastructure category, separate from vector DBs</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr"/>
+      <c r="G28" s="2" t="inlineStr"/>
+      <c r="H28" s="2" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>Highest Benchmark Performance</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>OMEGA (95.4% LongMemEval)</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>Zep (94.8% DMR / 71.2% LongMemEval)</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>OMEGA: #1 on LongMemEval; Zep: #1 on DMR; both outperform MemGPT</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>Memory benchmarks (LongMemEval, DMR) are becoming standardized evaluation criteria</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr"/>
+      <c r="G29" s="2" t="inlineStr"/>
+      <c r="H29" s="2" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>Most Production-Ready</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>Mem0</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>Zep</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>Mem0: exclusive AWS Agent SDK provider; Zep: 98% cost reduction, 90% latency reduction</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>Production deployment and cost efficiency are key differentiators, not just benchmark scores</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr"/>
+      <c r="G30" s="2" t="inlineStr"/>
+      <c r="H30" s="2" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>Best Open-Source / Local</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>OMEGA</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>Letta / MemGPT</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>OMEGA: fully local, zero dependencies, AES-256 encrypted; Letta: strong dev tooling</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>Privacy-first local memory is growing; developers want memory without cloud lock-in</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr"/>
+      <c r="G31" s="2" t="inlineStr"/>
+      <c r="H31" s="2" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>Vector DB Infrastructure</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>Pinecone ($750M, a16z-backed)</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>Weaviate ($200-500M+)</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>Pinecone: sub-33ms latency; Weaviate: open-source + self-hosted; Chroma: dev-friendly</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>Vector DBs remain foundational but purpose-built memory layers (Mem0, Zep, OMEGA) are emerging on top</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr"/>
+      <c r="G32" s="2" t="inlineStr"/>
+      <c r="H32" s="2" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>Biggest Paradigm Shift</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>Google Always On Memory Agent</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>SochDB (LLM-Native DB)</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>Google ditching vector DBs for LLM-driven SQLite memory; SochDB combining vector + SQL + token budgeting</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>The industry may be moving beyond vector databases toward LLM-native and hybrid memory architectures</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr"/>
+      <c r="G33" s="2" t="inlineStr"/>
+      <c r="H33" s="2" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="A18:H18"/>
+    <mergeCell ref="A26:H26"/>
+    <mergeCell ref="A11:H11"/>
+    <mergeCell ref="A1:H1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>